<commit_message>
Add question-level & by-school analysis + 5 visual charts
New sheet 'ניתוח שאלות ובתי ספר':
- Which sim questions best predict questionnaire score (Q4, Q3, Q8 lead)
- Per-school correlation breakdown (ranges -0.10 to 0.53)

New sheet 'גרפים' with 5 charts:
1. Correlation per dimension
2. Regression beta: AI vs no-AI grouped
3. Level distribution per question (% stacked)
4. Predictive power of each sim question
5. Sim-questionnaire correlation by school

https://claude.ai/code/session_011BCKSU8z4oQR3ER1cBLppb
</commit_message>
<xml_diff>
--- a/נתונים_מלאים_סימולציה_שאלון.xlsx
+++ b/נתונים_מלאים_סימולציה_שאלון.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="רגרסיה מרובה" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="השוואת AI מול ללא AI" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מיפוי ממדים" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ניתוח שאלות ובתי ספר" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="גרפים" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +64,27 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="14">
@@ -132,7 +155,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -155,11 +178,55 @@
       </bottom>
     </border>
     <border/>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
@@ -235,6 +302,53 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -309,6 +423,676 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>מתאם (r) בין סימולציה לשאלון, לפי ממד</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!U2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$3:$T$8</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$U$3:$U$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>r</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>מקדמי רגרסיה (β): עם AI מול ללא AI</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!U10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$11:$T$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$U$11:$U$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!V10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$11:$T$16</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$V$11:$V$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>β</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>התפלגות רמות לפי שאלה (%)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="percentStacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!U20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$21:$T$29</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$U$21:$U$29</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!V20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$21:$T$29</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$V$21:$V$29</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!W20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$21:$T$29</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$W$21:$W$29</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!X20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$21:$T$29</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$X$21:$X$29</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>אחוז</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>כוח ניבוי (r) של כל שאלת סימולציה את ציון השאלון</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!U32</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$33:$T$41</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$U$33:$U$41</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>מתאם סימולציה-שאלון לפי בית ספר (Top 12)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'גרפים'!U44</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'גרפים'!$T$45:$T$56</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'גרפים'!$U$45:$U$56</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -631,6 +1415,39 @@
           <t>נתוני כל תלמיד: ציוני סימולציה + ממדי שאלון פעלנות (תלמידי כיתה ז', N=1,235)</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="27" t="n"/>
+      <c r="K1" s="27" t="n"/>
+      <c r="L1" s="27" t="n"/>
+      <c r="M1" s="27" t="n"/>
+      <c r="N1" s="27" t="n"/>
+      <c r="O1" s="27" t="n"/>
+      <c r="P1" s="27" t="n"/>
+      <c r="Q1" s="27" t="n"/>
+      <c r="R1" s="27" t="n"/>
+      <c r="S1" s="27" t="n"/>
+      <c r="T1" s="27" t="n"/>
+      <c r="U1" s="27" t="n"/>
+      <c r="V1" s="27" t="n"/>
+      <c r="W1" s="27" t="n"/>
+      <c r="X1" s="27" t="n"/>
+      <c r="Y1" s="27" t="n"/>
+      <c r="Z1" s="27" t="n"/>
+      <c r="AA1" s="27" t="n"/>
+      <c r="AB1" s="27" t="n"/>
+      <c r="AC1" s="27" t="n"/>
+      <c r="AD1" s="27" t="n"/>
+      <c r="AE1" s="27" t="n"/>
+      <c r="AF1" s="27" t="n"/>
+      <c r="AG1" s="27" t="n"/>
+      <c r="AH1" s="28" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -84558,6 +85375,15 @@
           <t>סיכום אחוזים לפי רמה ולפי שאלה (מבוסס על תשובות מדשבורד)</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="28" t="n"/>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -85080,6 +85906,12 @@
           <t>מתאמי פירסון ושפירמן בין ממדי הסימולציה לממדי השאלון (N=1,235)</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="28" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -85361,6 +86193,13 @@
           <t>מטריצת מתאמים צולבת: כל ממד סימולציה מול כל ממד שאלון</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="28" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
@@ -85587,6 +86426,11 @@
           <t>רגרסיה מרובה: ניבוי ציון הסימולציה מ-6 ממדי השאלון</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="28" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -85594,6 +86438,11 @@
           <t>📊 ניתוח כלל המדגם  |  N=1223  |  R²=0.065 (6.5% ניבוי)  |  ציון ממוצע=2.05</t>
         </is>
       </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="28" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -85777,6 +86626,11 @@
           <t>🤖 קבוצת AI (פיילוט)  |  N=979  |  R²=0.058 (5.8% ניבוי)  |  ציון ממוצע=2.03</t>
         </is>
       </c>
+      <c r="B13" s="27" t="n"/>
+      <c r="C13" s="27" t="n"/>
+      <c r="D13" s="27" t="n"/>
+      <c r="E13" s="27" t="n"/>
+      <c r="F13" s="28" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -85960,6 +86814,11 @@
           <t>📝 קבוצת ללא AI (השוואה)  |  N=241  |  R²=0.130 (13.0% ניבוי)  |  ציון ממוצע=2.09</t>
         </is>
       </c>
+      <c r="B23" s="27" t="n"/>
+      <c r="C23" s="27" t="n"/>
+      <c r="D23" s="27" t="n"/>
+      <c r="E23" s="27" t="n"/>
+      <c r="F23" s="28" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -86169,6 +87028,9 @@
           <t>השוואת ביצוע בסימולציה: קבוצת AI מול קבוצת ללא AI</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="28" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -86431,6 +87293,9 @@
           <t>מיפוי: שאלות הסימולציה ↔ ממדי שאלון הפעלנות</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="28" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -86593,4 +87458,1334 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>אילו שאלות סימולציה מנבאות את ציון השאלון? + פילוח בתי ספר</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="30" t="inlineStr">
+        <is>
+          <t>חלק א': כוח הניבוי של כל שאלת סימולציה (N=1,202)</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="28" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>שאלה</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>נושא</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>r פשוט</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>β (תרומה ייחודית)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>מובהקות</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>יחידה חדשה</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="D5" s="33" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>אם תרגיש מתוסכל</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="D6" s="33" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>שיחה עם המורה</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>רגשות לגבי הציון</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>בעוד 3 שבועות</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>***</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>אם תתקע</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>למה קיבלת הציון</t>
+        </is>
+      </c>
+      <c r="C11" s="39" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+      <c r="D11" s="39" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="E11" s="39" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>איך תלמד</t>
+        </is>
+      </c>
+      <c r="C12" s="36" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>**</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>איך תדע שהדרך טובה</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="D13" s="39" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E13" s="39" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>מסקנה: Q4 (מוטיבציה עתידית), Q3 (ויסות רגשי) ו-Q8 (יחס לפידבק) הם המנבאים החזקים ביותר.</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="n"/>
+      <c r="C15" s="27" t="n"/>
+      <c r="D15" s="27" t="n"/>
+      <c r="E15" s="28" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>חלק ב': מתאם וביצוע לפי בית ספר (N≥30)</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="n"/>
+      <c r="C17" s="27" t="n"/>
+      <c r="D17" s="27" t="n"/>
+      <c r="E17" s="28" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>בית ספר</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>ממוצע סימולציה</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>ממוצע שאלון</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="inlineStr">
+        <is>
+          <t>תעופה וחלל ע"ש אלתרמן</t>
+        </is>
+      </c>
+      <c r="B19" s="39" t="n">
+        <v>67</v>
+      </c>
+      <c r="C19" s="39" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="D19" s="39" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E19" s="41" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>חט"ב שזר</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="n">
+        <v>90</v>
+      </c>
+      <c r="C20" s="36" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="D20" s="36" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="E20" s="41" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="38" t="inlineStr">
+        <is>
+          <t>חט"ב חדשה ברמות יצחק</t>
+        </is>
+      </c>
+      <c r="B21" s="39" t="n">
+        <v>44</v>
+      </c>
+      <c r="C21" s="39" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="D21" s="39" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="E21" s="41" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>חט"ב השרון</t>
+        </is>
+      </c>
+      <c r="B22" s="36" t="n">
+        <v>38</v>
+      </c>
+      <c r="C22" s="36" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="D22" s="36" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="E22" s="42" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="38" t="inlineStr">
+        <is>
+          <t>משה ארנס</t>
+        </is>
+      </c>
+      <c r="B23" s="39" t="n">
+        <v>66</v>
+      </c>
+      <c r="C23" s="39" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="D23" s="39" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="E23" s="41" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>המתמיד</t>
+        </is>
+      </c>
+      <c r="B24" s="36" t="n">
+        <v>58</v>
+      </c>
+      <c r="C24" s="36" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D24" s="36" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="E24" s="36" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="38" t="inlineStr">
+        <is>
+          <t>עתיד רזיאל</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="n">
+        <v>60</v>
+      </c>
+      <c r="C25" s="39" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="D25" s="39" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E25" s="39" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="35" t="inlineStr">
+        <is>
+          <t>יורם טהר-לב</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="n">
+        <v>65</v>
+      </c>
+      <c r="C26" s="36" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="D26" s="36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E26" s="36" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>חט"ב גוונים</t>
+        </is>
+      </c>
+      <c r="B27" s="39" t="n">
+        <v>82</v>
+      </c>
+      <c r="C27" s="39" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="D27" s="39" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E27" s="39" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="35" t="inlineStr">
+        <is>
+          <t>חט"ב שניה- רמות יצחק</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="n">
+        <v>73</v>
+      </c>
+      <c r="C28" s="36" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="D28" s="36" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E28" s="36" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="38" t="inlineStr">
+        <is>
+          <t>אורט עירוני ד</t>
+        </is>
+      </c>
+      <c r="B29" s="39" t="n">
+        <v>93</v>
+      </c>
+      <c r="C29" s="39" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="D29" s="39" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="E29" s="39" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="35" t="inlineStr">
+        <is>
+          <t>קמפוס פרס חדשנות ומנהיגות</t>
+        </is>
+      </c>
+      <c r="B30" s="36" t="n">
+        <v>43</v>
+      </c>
+      <c r="C30" s="36" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="D30" s="36" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E30" s="36" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>אורט גרינברג קריית טבעון</t>
+        </is>
+      </c>
+      <c r="B31" s="39" t="n">
+        <v>49</v>
+      </c>
+      <c r="C31" s="39" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="D31" s="39" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="E31" s="39" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="35" t="inlineStr">
+        <is>
+          <t>צין</t>
+        </is>
+      </c>
+      <c r="B32" s="36" t="n">
+        <v>36</v>
+      </c>
+      <c r="C32" s="36" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="D32" s="36" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E32" s="36" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="38" t="inlineStr">
+        <is>
+          <t>חטיבת בארי</t>
+        </is>
+      </c>
+      <c r="B33" s="39" t="n">
+        <v>95</v>
+      </c>
+      <c r="C33" s="39" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="D33" s="39" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="E33" s="39" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="35" t="inlineStr">
+        <is>
+          <t>עמל דקל וילנאי</t>
+        </is>
+      </c>
+      <c r="B34" s="36" t="n">
+        <v>50</v>
+      </c>
+      <c r="C34" s="36" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="D34" s="36" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="E34" s="41" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="inlineStr">
+        <is>
+          <t>ישיבה תיכונית חדשה</t>
+        </is>
+      </c>
+      <c r="B35" s="39" t="n">
+        <v>51</v>
+      </c>
+      <c r="C35" s="39" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="D35" s="39" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="E35" s="42" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>הלל</t>
+        </is>
+      </c>
+      <c r="B36" s="36" t="n">
+        <v>32</v>
+      </c>
+      <c r="C36" s="36" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="D36" s="36" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="E36" s="42" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="inlineStr">
+        <is>
+          <t>ישיבה תיכונית אמי"ת אלירז</t>
+        </is>
+      </c>
+      <c r="B37" s="39" t="n">
+        <v>40</v>
+      </c>
+      <c r="C37" s="39" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="D37" s="39" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="E37" s="39" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="40" t="inlineStr">
+        <is>
+          <t>שים לב: המתאם משתנה מאוד בין בתי ספר (0.10- עד 0.53), המעיד על השפעת הקשר החינוכי.</t>
+        </is>
+      </c>
+      <c r="B39" s="27" t="n"/>
+      <c r="C39" s="27" t="n"/>
+      <c r="D39" s="27" t="n"/>
+      <c r="E39" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
+    <col hidden="1" width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="13" customWidth="1" min="22" max="22"/>
+    <col hidden="1" width="13" customWidth="1" min="23" max="23"/>
+    <col hidden="1" width="13" customWidth="1" min="24" max="24"/>
+    <col hidden="1" width="13" customWidth="1" min="25" max="25"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="43" t="inlineStr">
+        <is>
+          <t>גרפים ויזואליים</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="T2" s="39" t="inlineStr">
+        <is>
+          <t>ממד</t>
+        </is>
+      </c>
+      <c r="U2" s="39" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="T3" s="39" t="inlineStr">
+        <is>
+          <t>מוטיבציה</t>
+        </is>
+      </c>
+      <c r="U3" s="39" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="T4" s="39" t="inlineStr">
+        <is>
+          <t>תודעת צמיחה</t>
+        </is>
+      </c>
+      <c r="U4" s="39" t="n">
+        <v>0.064</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="T5" s="39" t="inlineStr">
+        <is>
+          <t>יוזמה</t>
+        </is>
+      </c>
+      <c r="U5" s="39" t="n">
+        <v>0.126</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="T6" s="39" t="inlineStr">
+        <is>
+          <t>ויסות</t>
+        </is>
+      </c>
+      <c r="U6" s="39" t="n">
+        <v>0.124</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="T7" s="39" t="inlineStr">
+        <is>
+          <t>מודעות</t>
+        </is>
+      </c>
+      <c r="U7" s="39" t="n">
+        <v>0.041</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="T8" s="39" t="inlineStr">
+        <is>
+          <t>תמיכה</t>
+        </is>
+      </c>
+      <c r="U8" s="39" t="n">
+        <v>0.131</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="T10" s="39" t="inlineStr">
+        <is>
+          <t>ממד</t>
+        </is>
+      </c>
+      <c r="U10" s="39" t="inlineStr">
+        <is>
+          <t>עם AI</t>
+        </is>
+      </c>
+      <c r="V10" s="39" t="inlineStr">
+        <is>
+          <t>ללא AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="T11" s="39" t="inlineStr">
+        <is>
+          <t>מוטיבציה</t>
+        </is>
+      </c>
+      <c r="U11" s="39" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="V11" s="39" t="n">
+        <v>0.259</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="T12" s="39" t="inlineStr">
+        <is>
+          <t>תודעת צמיחה</t>
+        </is>
+      </c>
+      <c r="U12" s="39" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="V12" s="39" t="n">
+        <v>0.161</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="T13" s="39" t="inlineStr">
+        <is>
+          <t>יוזמה</t>
+        </is>
+      </c>
+      <c r="U13" s="39" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="V13" s="39" t="n">
+        <v>0.049</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="T14" s="39" t="inlineStr">
+        <is>
+          <t>ויסות</t>
+        </is>
+      </c>
+      <c r="U14" s="39" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="V14" s="39" t="n">
+        <v>-0.148</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="T15" s="39" t="inlineStr">
+        <is>
+          <t>מודעות</t>
+        </is>
+      </c>
+      <c r="U15" s="39" t="n">
+        <v>-0.017</v>
+      </c>
+      <c r="V15" s="39" t="n">
+        <v>0.082</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="T16" s="39" t="inlineStr">
+        <is>
+          <t>תמיכה</t>
+        </is>
+      </c>
+      <c r="U16" s="39" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="V16" s="39" t="n">
+        <v>-0.011</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="T20" s="39" t="inlineStr">
+        <is>
+          <t>שאלה</t>
+        </is>
+      </c>
+      <c r="U20" s="39" t="inlineStr">
+        <is>
+          <t>רמה 1</t>
+        </is>
+      </c>
+      <c r="V20" s="39" t="inlineStr">
+        <is>
+          <t>רמה 2</t>
+        </is>
+      </c>
+      <c r="W20" s="39" t="inlineStr">
+        <is>
+          <t>רמה 3</t>
+        </is>
+      </c>
+      <c r="X20" s="39" t="inlineStr">
+        <is>
+          <t>רמה 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="T21" s="39" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="U21" s="39" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="V21" s="39" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="W21" s="39" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="X21" s="39" t="n">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="T22" s="39" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="U22" s="39" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="V22" s="39" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="W22" s="39" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="X22" s="39" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="T23" s="39" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="U23" s="39" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="V23" s="39" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="W23" s="39" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="X23" s="39" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="T24" s="39" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="U24" s="39" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="V24" s="39" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="W24" s="39" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="X24" s="39" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="T25" s="39" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="U25" s="39" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="V25" s="39" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="W25" s="39" t="n">
+        <v>22</v>
+      </c>
+      <c r="X25" s="39" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="T26" s="39" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="U26" s="39" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="V26" s="39" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="W26" s="39" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="X26" s="39" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="T27" s="39" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="U27" s="39" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="V27" s="39" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="W27" s="39" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="X27" s="39" t="n">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="T28" s="39" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="U28" s="39" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="V28" s="39" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="W28" s="39" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="X28" s="39" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="T29" s="39" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="U29" s="39" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="V29" s="39" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="W29" s="39" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="X29" s="39" t="n">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="T32" s="39" t="inlineStr">
+        <is>
+          <t>שאלה</t>
+        </is>
+      </c>
+      <c r="U32" s="39" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="T33" s="39" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="U33" s="39" t="n">
+        <v>0.177</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="T34" s="39" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="U34" s="39" t="n">
+        <v>0.164</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="T35" s="39" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="U35" s="39" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="T36" s="39" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="U36" s="39" t="n">
+        <v>0.119</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="T37" s="39" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="U37" s="39" t="n">
+        <v>0.112</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="T38" s="39" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="U38" s="39" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="T39" s="39" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="U39" s="39" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="T40" s="39" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="U40" s="39" t="n">
+        <v>0.079</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="T41" s="39" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="U41" s="39" t="n">
+        <v>0.047</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="T44" s="39" t="inlineStr">
+        <is>
+          <t>בית ספר</t>
+        </is>
+      </c>
+      <c r="U44" s="39" t="inlineStr">
+        <is>
+          <t>מתאם r</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="T45" s="39" t="inlineStr">
+        <is>
+          <t>משה ארנס</t>
+        </is>
+      </c>
+      <c r="U45" s="39" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="T46" s="39" t="inlineStr">
+        <is>
+          <t>חט"ב חדשה ברמות יצ</t>
+        </is>
+      </c>
+      <c r="U46" s="39" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="T47" s="39" t="inlineStr">
+        <is>
+          <t>עמל דקל וילנאי</t>
+        </is>
+      </c>
+      <c r="U47" s="39" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="T48" s="39" t="inlineStr">
+        <is>
+          <t>חט"ב שזר</t>
+        </is>
+      </c>
+      <c r="U48" s="39" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="T49" s="39" t="inlineStr">
+        <is>
+          <t>תעופה וחלל ע"ש אלת</t>
+        </is>
+      </c>
+      <c r="U49" s="39" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="T50" s="39" t="inlineStr">
+        <is>
+          <t>המתמיד</t>
+        </is>
+      </c>
+      <c r="U50" s="39" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="T51" s="39" t="inlineStr">
+        <is>
+          <t>חט"ב גוונים</t>
+        </is>
+      </c>
+      <c r="U51" s="39" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="T52" s="39" t="inlineStr">
+        <is>
+          <t>חט"ב שניה- רמות יצ</t>
+        </is>
+      </c>
+      <c r="U52" s="39" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="T53" s="39" t="inlineStr">
+        <is>
+          <t>חטיבת בארי</t>
+        </is>
+      </c>
+      <c r="U53" s="39" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="T54" s="39" t="inlineStr">
+        <is>
+          <t>יורם טהר-לב</t>
+        </is>
+      </c>
+      <c r="U54" s="39" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="T55" s="39" t="inlineStr">
+        <is>
+          <t>אורט עירוני ד</t>
+        </is>
+      </c>
+      <c r="U55" s="39" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="T56" s="39" t="inlineStr">
+        <is>
+          <t>צין</t>
+        </is>
+      </c>
+      <c r="U56" s="39" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add school-level characterization: what drives sim-questionnaire alignment
New sheet 'מאפייני בתי ספר' comparing high-r vs low-r schools:
- High-r schools: 70% AI usage; low-r schools: 85% AI usage
- Nearly all zero/negative-r schools have 100% AI saturation
- School size predicts r strength (reliability artifact, r=.46*)
- %AI negatively associated with r (r=-.37) - reinforces main thesis
Includes caveat: only 19 schools, trend-level evidence.

https://claude.ai/code/session_011BCKSU8z4oQR3ER1cBLppb
</commit_message>
<xml_diff>
--- a/נתונים_מלאים_סימולציה_שאלון.xlsx
+++ b/נתונים_מלאים_סימולציה_שאלון.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מיפוי ממדים" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ניתוח שאלות ובתי ספר" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="גרפים" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאפייני בתי ספר" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,6 +86,12 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="14">
@@ -226,7 +233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
@@ -348,6 +355,60 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1410,7 +1471,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>נתוני כל תלמיד: ציוני סימולציה + ממדי שאלון פעלנות (תלמידי כיתה ז', N=1,235)</t>
         </is>
@@ -85348,6 +85409,1065 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="44" t="inlineStr">
+        <is>
+          <t>מה מאפיין בתי ספר עם מתאם גבוה מול נמוך בין דיווח לביצוע?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>השוואת קבוצות קיצון (שליש עליון מול שליש תחתון, 6 בתי ספר בכל קבוצה)</t>
+        </is>
+      </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="27" t="n"/>
+      <c r="E3" s="27" t="n"/>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="28" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>מאפיין</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>🟢 מתאם גבוה</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>🔴 מתאם נמוך</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>הפרש</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="46" t="inlineStr">
+        <is>
+          <t>r ממוצע</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="inlineStr">
+        <is>
+          <t>0.41</t>
+        </is>
+      </c>
+      <c r="C5" s="47" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="D5" s="47" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="48" t="inlineStr">
+        <is>
+          <t>גודל בית ספר (N)</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="C6" s="49" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D6" s="49" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>ממוצע סימולציה</t>
+        </is>
+      </c>
+      <c r="B7" s="47" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="C7" s="47" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="D7" s="47" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="48" t="inlineStr">
+        <is>
+          <t>שונות סימולציה (SD)</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+      <c r="C8" s="49" t="inlineStr">
+        <is>
+          <t>0.29</t>
+        </is>
+      </c>
+      <c r="D8" s="49" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>ממוצע שאלון</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="inlineStr">
+        <is>
+          <t>3.60</t>
+        </is>
+      </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>3.53</t>
+        </is>
+      </c>
+      <c r="D9" s="47" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="48" t="inlineStr">
+        <is>
+          <t>שונות שאלון (SD)</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>0.49</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="D10" s="49" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>% שימוש ב-AI</t>
+        </is>
+      </c>
+      <c r="B11" s="50" t="inlineStr">
+        <is>
+          <t>70%</t>
+        </is>
+      </c>
+      <c r="C11" s="51" t="inlineStr">
+        <is>
+          <t>85%</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t>-15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="45" t="inlineStr">
+        <is>
+          <t>מה מנבא את עוצמת המתאם ברמת בית הספר? (מתאם בין מאפיין ל-r, 19 בתי ספר)</t>
+        </is>
+      </c>
+      <c r="B14" s="27" t="n"/>
+      <c r="C14" s="27" t="n"/>
+      <c r="D14" s="27" t="n"/>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="28" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>מאפיין</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>מתאם עם r</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>פרשנות</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="48" t="inlineStr">
+        <is>
+          <t>גודל בית ספר</t>
+        </is>
+      </c>
+      <c r="B16" s="52" t="inlineStr">
+        <is>
+          <t>+0.459 *</t>
+        </is>
+      </c>
+      <c r="C16" s="49" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="D16" s="53" t="inlineStr">
+        <is>
+          <t>בתי ספר גדולים → מתאם חזק (ככל הנראה אפקט מהימנות)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="46" t="inlineStr">
+        <is>
+          <t>ממוצע סימולציה</t>
+        </is>
+      </c>
+      <c r="B17" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+0.444 </t>
+        </is>
+      </c>
+      <c r="C17" s="47" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="D17" s="54" t="inlineStr">
+        <is>
+          <t>ביצוע גבוה יותר → התאמה טובה יותר</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="48" t="inlineStr">
+        <is>
+          <t>% שימוש ב-AI</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-0.372 </t>
+        </is>
+      </c>
+      <c r="C18" s="49" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="D18" s="53" t="inlineStr">
+        <is>
+          <t>יותר AI → מתאם חלש יותר (תומך בהשערה!)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="46" t="inlineStr">
+        <is>
+          <t>שונות שאלון</t>
+        </is>
+      </c>
+      <c r="B19" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+0.425 </t>
+        </is>
+      </c>
+      <c r="C19" s="47" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="D19" s="54" t="inlineStr">
+        <is>
+          <t>פיזור גדול יותר בשאלון → מתאם חזק יותר</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="48" t="inlineStr">
+        <is>
+          <t>ממוצע שאלון</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+0.161 </t>
+        </is>
+      </c>
+      <c r="C20" s="49" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="D20" s="53" t="inlineStr">
+        <is>
+          <t>אין קשר ברור</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="46" t="inlineStr">
+        <is>
+          <t>שונות סימולציה</t>
+        </is>
+      </c>
+      <c r="B21" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+0.199 </t>
+        </is>
+      </c>
+      <c r="C21" s="47" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="D21" s="54" t="inlineStr">
+        <is>
+          <t>אין קשר ברור</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>טבלה מלאה: כל בתי הספר (N≥30), ממוין לפי מתאם</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="n"/>
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="27" t="n"/>
+      <c r="E24" s="27" t="n"/>
+      <c r="F24" s="27" t="n"/>
+      <c r="G24" s="28" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>בית ספר</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>ממוצע
+סים</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>SD
+סים</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>ממוצע
+שאלון</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>%
+AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="55" t="inlineStr">
+        <is>
+          <t>משה ארנס</t>
+        </is>
+      </c>
+      <c r="B26" s="50" t="n">
+        <v>66</v>
+      </c>
+      <c r="C26" s="56" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D26" s="50" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="E26" s="50" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F26" s="50" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="G26" s="50" t="inlineStr">
+        <is>
+          <t>74%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="55" t="inlineStr">
+        <is>
+          <t>חט"ב חדשה ברמות יצחק</t>
+        </is>
+      </c>
+      <c r="B27" s="50" t="n">
+        <v>44</v>
+      </c>
+      <c r="C27" s="56" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D27" s="50" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="E27" s="50" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F27" s="50" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="G27" s="50" t="inlineStr">
+        <is>
+          <t>43%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="55" t="inlineStr">
+        <is>
+          <t>עמל דקל וילנאי</t>
+        </is>
+      </c>
+      <c r="B28" s="50" t="n">
+        <v>50</v>
+      </c>
+      <c r="C28" s="56" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D28" s="50" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="E28" s="50" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F28" s="50" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="G28" s="50" t="inlineStr">
+        <is>
+          <t>72%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="55" t="inlineStr">
+        <is>
+          <t>חט"ב שזר</t>
+        </is>
+      </c>
+      <c r="B29" s="50" t="n">
+        <v>90</v>
+      </c>
+      <c r="C29" s="56" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D29" s="50" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="E29" s="50" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F29" s="50" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="G29" s="50" t="inlineStr">
+        <is>
+          <t>59%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="55" t="inlineStr">
+        <is>
+          <t>תעופה וחלל ע"ש אלתרמן</t>
+        </is>
+      </c>
+      <c r="B30" s="50" t="n">
+        <v>67</v>
+      </c>
+      <c r="C30" s="56" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D30" s="50" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="E30" s="50" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F30" s="50" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G30" s="50" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="54" t="inlineStr">
+        <is>
+          <t>המתמיד</t>
+        </is>
+      </c>
+      <c r="B31" s="47" t="n">
+        <v>58</v>
+      </c>
+      <c r="C31" s="57" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D31" s="47" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E31" s="47" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="F31" s="47" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="G31" s="47" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="53" t="inlineStr">
+        <is>
+          <t>חט"ב גוונים</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="n">
+        <v>82</v>
+      </c>
+      <c r="C32" s="58" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D32" s="49" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="E32" s="49" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F32" s="49" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G32" s="49" t="inlineStr">
+        <is>
+          <t>66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="54" t="inlineStr">
+        <is>
+          <t>חט"ב שניה- רמות יצחק</t>
+        </is>
+      </c>
+      <c r="B33" s="47" t="n">
+        <v>73</v>
+      </c>
+      <c r="C33" s="57" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D33" s="47" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="E33" s="47" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F33" s="47" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G33" s="47" t="inlineStr">
+        <is>
+          <t>67%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="53" t="inlineStr">
+        <is>
+          <t>חטיבת בארי</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="n">
+        <v>95</v>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D34" s="49" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="E34" s="49" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F34" s="49" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="G34" s="49" t="inlineStr">
+        <is>
+          <t>68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="54" t="inlineStr">
+        <is>
+          <t>יורם טהר-לב</t>
+        </is>
+      </c>
+      <c r="B35" s="47" t="n">
+        <v>65</v>
+      </c>
+      <c r="C35" s="57" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D35" s="47" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="E35" s="47" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F35" s="47" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G35" s="47" t="inlineStr">
+        <is>
+          <t>98%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="53" t="inlineStr">
+        <is>
+          <t>אורט עירוני ד</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="n">
+        <v>93</v>
+      </c>
+      <c r="C36" s="58" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D36" s="49" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E36" s="49" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F36" s="49" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="G36" s="49" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="54" t="inlineStr">
+        <is>
+          <t>צין</t>
+        </is>
+      </c>
+      <c r="B37" s="47" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" s="57" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D37" s="47" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="E37" s="47" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F37" s="47" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="G37" s="47" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="53" t="inlineStr">
+        <is>
+          <t>ישיבה תיכונית אמי"ת אלירז</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="n">
+        <v>40</v>
+      </c>
+      <c r="C38" s="58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D38" s="49" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="E38" s="49" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F38" s="49" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="G38" s="49" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="54" t="inlineStr">
+        <is>
+          <t>אורט גרינברג קריית טבעון</t>
+        </is>
+      </c>
+      <c r="B39" s="47" t="n">
+        <v>49</v>
+      </c>
+      <c r="C39" s="57" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D39" s="47" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="E39" s="47" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F39" s="47" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="G39" s="47" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="53" t="inlineStr">
+        <is>
+          <t>קמפוס פרס חדשנות ומנהיגות</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="n">
+        <v>43</v>
+      </c>
+      <c r="C40" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D40" s="49" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="E40" s="49" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F40" s="49" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G40" s="49" t="inlineStr">
+        <is>
+          <t>53%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="54" t="inlineStr">
+        <is>
+          <t>עתיד רזיאל</t>
+        </is>
+      </c>
+      <c r="B41" s="47" t="n">
+        <v>60</v>
+      </c>
+      <c r="C41" s="57" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D41" s="47" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="E41" s="47" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F41" s="47" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G41" s="47" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="59" t="inlineStr">
+        <is>
+          <t>ישיבה תיכונית חדשה</t>
+        </is>
+      </c>
+      <c r="B42" s="51" t="n">
+        <v>51</v>
+      </c>
+      <c r="C42" s="60" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="D42" s="51" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="E42" s="51" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="F42" s="51" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="G42" s="51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="59" t="inlineStr">
+        <is>
+          <t>הלל</t>
+        </is>
+      </c>
+      <c r="B43" s="51" t="n">
+        <v>32</v>
+      </c>
+      <c r="C43" s="60" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="D43" s="51" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="E43" s="51" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F43" s="51" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="G43" s="51" t="inlineStr">
+        <is>
+          <t>56%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="59" t="inlineStr">
+        <is>
+          <t>חט"ב השרון</t>
+        </is>
+      </c>
+      <c r="B44" s="51" t="n">
+        <v>38</v>
+      </c>
+      <c r="C44" s="60" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="D44" s="51" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="E44" s="51" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F44" s="51" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="G44" s="51" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="61" t="inlineStr">
+        <is>
+          <t>מסקנות מרכזיות:</t>
+        </is>
+      </c>
+      <c r="B46" s="27" t="n"/>
+      <c r="C46" s="27" t="n"/>
+      <c r="D46" s="27" t="n"/>
+      <c r="E46" s="27" t="n"/>
+      <c r="F46" s="27" t="n"/>
+      <c r="G46" s="28" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="46" t="inlineStr">
+        <is>
+          <t>1. בתי ספר עם שימוש נמוך יותר ב-AI (70%) מראים מתאם חזק יותר מאלה עם שימוש גבוה (85%) —</t>
+        </is>
+      </c>
+      <c r="B47" s="27" t="n"/>
+      <c r="C47" s="27" t="n"/>
+      <c r="D47" s="27" t="n"/>
+      <c r="E47" s="27" t="n"/>
+      <c r="F47" s="27" t="n"/>
+      <c r="G47" s="28" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   חיזוק ברמת בית הספר להשערה שה-AI ממתן את הקשר בין דיווח עצמי לביצוע.</t>
+        </is>
+      </c>
+      <c r="B48" s="27" t="n"/>
+      <c r="C48" s="27" t="n"/>
+      <c r="D48" s="27" t="n"/>
+      <c r="E48" s="27" t="n"/>
+      <c r="F48" s="27" t="n"/>
+      <c r="G48" s="28" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="54" t="inlineStr">
+        <is>
+          <t>2. כמעט כל בתי הספר עם מתאם אפסי/שלילי הם בעלי 100% שימוש ב-AI</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="n"/>
+      <c r="C49" s="27" t="n"/>
+      <c r="D49" s="27" t="n"/>
+      <c r="E49" s="27" t="n"/>
+      <c r="F49" s="27" t="n"/>
+      <c r="G49" s="28" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (חט"ב השרון, עתיד רזיאל, ישיבה תיכונית חדשה, צין, אורט גרינברג, אמי"ת אלירז).</t>
+        </is>
+      </c>
+      <c r="B50" s="27" t="n"/>
+      <c r="C50" s="27" t="n"/>
+      <c r="D50" s="27" t="n"/>
+      <c r="E50" s="27" t="n"/>
+      <c r="F50" s="27" t="n"/>
+      <c r="G50" s="28" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="54" t="inlineStr">
+        <is>
+          <t>3. בתי ספר גדולים יותר מראים מתאם יציב יותר (אפקט מהימנות סטטיסטי).</t>
+        </is>
+      </c>
+      <c r="B51" s="27" t="n"/>
+      <c r="C51" s="27" t="n"/>
+      <c r="D51" s="27" t="n"/>
+      <c r="E51" s="27" t="n"/>
+      <c r="F51" s="27" t="n"/>
+      <c r="G51" s="28" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="54" t="inlineStr">
+        <is>
+          <t>4. אזהרה: הניתוח מבוסס על 19 בתי ספר בלבד, ולכן המתאמים ברמת בית הספר מעידים על מגמה</t>
+        </is>
+      </c>
+      <c r="B52" s="27" t="n"/>
+      <c r="C52" s="27" t="n"/>
+      <c r="D52" s="27" t="n"/>
+      <c r="E52" s="27" t="n"/>
+      <c r="F52" s="27" t="n"/>
+      <c r="G52" s="28" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ולא על קשר מבוסס. נדרשת זהירות בהכללה.</t>
+        </is>
+      </c>
+      <c r="B53" s="27" t="n"/>
+      <c r="C53" s="27" t="n"/>
+      <c r="D53" s="27" t="n"/>
+      <c r="E53" s="27" t="n"/>
+      <c r="F53" s="27" t="n"/>
+      <c r="G53" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A52:G52"/>
+    <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A46:G46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -85370,7 +86490,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>סיכום אחוזים לפי רמה ולפי שאלה (מבוסס על תשובות מדשבורד)</t>
         </is>
@@ -85901,7 +87021,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>מתאמי פירסון ושפירמן בין ממדי הסימולציה לממדי השאלון (N=1,235)</t>
         </is>
@@ -86188,7 +87308,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>מטריצת מתאמים צולבת: כל ממד סימולציה מול כל ממד שאלון</t>
         </is>
@@ -86421,7 +87541,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>רגרסיה מרובה: ניבוי ציון הסימולציה מ-6 ממדי השאלון</t>
         </is>
@@ -87023,7 +88143,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>השוואת ביצוע בסימולציה: קבוצת AI מול קבוצת ללא AI</t>
         </is>
@@ -87288,7 +88408,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>מיפוי: שאלות הסימולציה ↔ ממדי שאלון הפעלנות</t>
         </is>
@@ -87482,6 +88602,10 @@
           <t>אילו שאלות סימולציה מנבאות את ציון השאלון? + פילוח בתי ספר</t>
         </is>
       </c>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="28" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="30" t="inlineStr">

</xml_diff>